<commit_message>
Update backend, redis and frontend changes
</commit_message>
<xml_diff>
--- a/backend/data/New Flagged FAQ.xlsx
+++ b/backend/data/New Flagged FAQ.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG5"/>
+  <dimension ref="A1:AG6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -978,14 +978,11 @@
           <t>pending</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
           <t>modify</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr">
         <is>
           <t>medium</t>
@@ -1001,21 +998,164 @@
           <t>Show opening stock for buyer for the requested quantity month</t>
         </is>
       </c>
-      <c r="Y5" t="inlineStr"/>
-      <c r="Z5" t="inlineStr"/>
-      <c r="AA5" t="inlineStr"/>
       <c r="AB5" t="b">
         <v>1</v>
       </c>
-      <c r="AC5" t="inlineStr"/>
-      <c r="AD5" t="inlineStr"/>
       <c r="AE5" t="inlineStr">
         <is>
           <t>feedback</t>
         </is>
       </c>
-      <c r="AF5" t="inlineStr"/>
-      <c r="AG5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>8731ca2d75cb1b200bd9d6d83447fb01ac15cf6a7fe684a2f1d0a86639b3c881</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-10-13T10:23:15.736910+00:00</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Docket Employee Report</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>performance index more</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>performance_index</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>performance_index</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>[{"name": "performance_index", "value": "10", "source": "input"}, {"name": "employee_org", "value": "ACD - PRODUCTS", "source": "option"}, {"name": "period_type", "value": "Month", "source": "option"}, {"name": "period_name", "value": "APR-24", "source": "option"}]</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>SELECT TNO, ENAME, EMP_DEPT, EMP_ORG_NAME, PERIOD_NAME, PERFORMANCE_INDEX FROM KPCL_REPORTING.KPC_FULL_KIT_DOCKET_EMP WHERE ((PERFORMANCE_INDEX &gt; {performance_index} AND KPC_FULL_KIT_DOCKET_EMP.EMP_ORG_NAME LIKE '%{employee_org}%') AND KPC_FULL_KIT_DOCKET_EMP.PERIOD_TYPE LIKE '%{period_type}%') AND KPC_FULL_KIT_DOCKET_EMP.PERIOD_NAME LIKE '%{period_name}%' ORDER BY PERFORMANCE_INDEX DESC;</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>SELECT TNO, ENAME, EMP_DEPT, EMP_ORG_NAME, PERIOD_NAME, PERFORMANCE_INDEX FROM KPCL_REPORTING.KPC_FULL_KIT_DOCKET_EMP WHERE ((PERFORMANCE_INDEX &gt; 10 AND KPC_FULL_KIT_DOCKET_EMP.EMP_ORG_NAME LIKE '%ACD - PRODUCTS%') AND KPC_FULL_KIT_DOCKET_EMP.PERIOD_TYPE LIKE '%Month%') AND KPC_FULL_KIT_DOCKET_EMP.PERIOD_NAME LIKE '%APR-24%' ORDER BY PERFORMANCE_INDEX DESC;</t>
+        </is>
+      </c>
+      <c r="M6" t="n">
+        <v>47</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>445c24bc-1267-4e36-aa62-85d4dbaa8c46</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>d4ed35c0-6079-4c57-a815-f15ef2d2d9d8</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>426bdc74-29e8-45e6-b88a-7020c0f4a0c3</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>thumbs_up</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>up</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>/performance_index {10} more</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>performance index more</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>reuse</t>
+        </is>
+      </c>
+      <c r="Z6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB6" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>[{"TNO": 40394, "ENAME": "SANKET X BHOITE", "EMP_DEPT": "Manufacturing-Machin", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 108.09}, {"TNO": 40396, "ENAME": "RAJESH VITTHAL KUTE", "EMP_DEPT": "Manufacturing-Machin", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 103.18}, {"TNO": 40357, "ENAME": "DANISH DASTAGIR KAZI", "EMP_DEPT": "Manufacturing-Machin", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 100.88}, {"TNO": 40517, "ENAME": "NAGESH JAGANNATH BORAMANI", "EMP_DEPT": "Manufacturing-Machin", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 100.28}, {"TNO": 30373, "ENAME": "AVDHUT MARUTI DESAI", "EMP_DEPT": "Manufacturing-Assemb", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 100}, {"TNO": 40215, "ENAME": "AKSHAY ROHIDAS LADKAT", "EMP_DEPT": "Manufacturing-Machin", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 99.4}, {"TNO": 93262, "ENAME": "ATIF ASLAM MANER", "EMP_DEPT": "Manufacturing-Machin", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 97.63}, {"TNO": 40186, "ENAME": "NIKHIL UTTAM KAMBALE", "EMP_DEPT": "Manufacturing-Machin", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 96.87}, {"TNO": 93284, "ENAME": "AKASH KASHINATH NILAJI", "EMP_DEPT": "Manufacturing-Machin", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 96.71}, {"TNO": 40229, "ENAME": "SHUBHAM CHAGAN KHOT", "EMP_DEPT": "Manufacturing-Machin", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 96.27}, {"TNO": 40395, "ENAME": "LAXMAN VITTHAL PAWAR", "EMP_DEPT": "Manufacturing-Machin", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 95.86}, {"TNO": 40188, "ENAME": "SHRIKANT CHANDRKANT YADAV", "EMP_DEPT": "Manufacturing-Machin", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 95.29}, {"TNO": 40560, "ENAME": "SIDHESH SATISH GURAV", "EMP_DEPT": "Manufacturing-Assemb", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 94.72}, {"TNO": 40200, "ENAME": "SANDIP DATTATRAY MHASKE", "EMP_DEPT": "Manufacturing-Machin", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 93.95}, {"TNO": 40115, "ENAME": "RAHUL ISHWAR SHELAKE", "EMP_DEPT": "Manufacturing-Machin", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 93.8}, {"TNO": 40480, "ENAME": "MITHUN MASKU DOMBALE", "EMP_DEPT": "Manufacturing-Assemb", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 92.86}, {"TNO": 40217, "ENAME": "ROHIT VIJAY KAMBLE", "EMP_DEPT": "Manufacturing-Assemb", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 92.23}, {"TNO": 40169, "ENAME": "AMOL RAJU GAIKWAD", "EMP_DEPT": "Manufacturing-Machin", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 92.14}, {"TNO": 40295, "ENAME": "MANGESH CHANDRAKANT SAWANT", "EMP_DEPT": "Manufacturing-Assemb", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 91.33}, {"TNO": 40521, "ENAME": "AMOL  MORE", "EMP_DEPT": "Manufacturing-Machin", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 89.92}, {"TNO": 40249, "ENAME": "ROHIT SARJERAO PATIL", "EMP_DEPT": "Manufacturing-Machin", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 89.25}, {"TNO": 40475, "ENAME": "AKSHAY VITTHAL KAMBLE", "EMP_DEPT": "Manufacturing-Assemb", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 88.6}, {"TNO": 11791, "ENAME": "ROHIT JAYKAR PATIL", "EMP_DEPT": "Manufacturing-Machin", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 88.2}, {"TNO": 40183, "ENAME": "SHUBHAM KONDIBA DALVI", "EMP_DEPT": "Manufacturing-Machin", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 87.89}, {"TNO": 40564, "ENAME": "PRAJWAL PATALU ADISARE", "EMP_DEPT": "Manufacturing-Assemb", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 87.66}, {"TNO": 11589, "ENAME": "ASLAM NABILAL SHAIKH", "EMP_DEPT": "Manufacturing-Machin", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 87.59}, {"TNO": 40358, "ENAME": "SAGAR BHIMRAO NIVEKAR", "EMP_DEPT": "Manufacturing-Machin", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 87.52}, {"TNO": 40156, "ENAME": "BALAJI BALVANT YEDKE", "EMP_DEPT": "Manufacturing-Machin", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 87.38}, {"TNO": 40189, "ENAME": "HANUMANT ROHIDAS RAUT", "EMP_DEPT": "Manufacturing-Machin", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 86.65}, {"TNO": 11790, "ENAME": "MARUTI MAHADEV BHOSALE", "EMP_DEPT": "Manufacturing-Machin", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 85.38}, {"TNO": 40207, "ENAME": "HARSHAD BALASAHEB JAGTAP", "EMP_DEPT": "Manufacturing-Machin", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 84.78}, {"TNO": 40397, "ENAME": "BALASAHEB PRABHAKAR MOTHERAO", "EMP_DEPT": "Manufacturing-Machin", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 84.59}, {"TNO": 40474, "ENAME": "SUSHANT ANUPKUMAR GUPTA", "EMP_DEPT": "Manufacturing-Assemb", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 84.08}, {"TNO": 40191, "ENAME": "BAPU DATTATRAYA SONAWALE", "EMP_DEPT": "Manufacturing-Machin", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 83.29}, {"TNO": 40244, "ENAME": "SHUBHAM SANJAYPRASAD TIWARI", "EMP_DEPT": "Manufacturing-Machin", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 82.75}, {"TNO": 40211, "ENAME": "PRAMOD KUMAR GIRAJ SINGH", "EMP_DEPT": "Manufacturing-Machin", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 81.98}, {"TNO": 40502, "ENAME": "DILIPKUMAR . MOHE", "EMP_DEPT": "Manufacturing-Machin", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 81.34}, {"TNO": 40214, "ENAME": "NIKHIL BHAUSO ZITE", "EMP_DEPT": "Manufacturing-Machin", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 81.3}, {"TNO": 40393, "ENAME": "GANESH SURESH JADHAV", "EMP_DEPT": "Manufacturing-Machin", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 79.83}, {"TNO": 40230, "ENAME": "SHUBHAM BHAGWAN TODKAR", "EMP_DEPT": "Manufacturing-Machin", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 79.6}, {"TNO": 40195, "ENAME": "PUSHKAR KISAN BARNE", "EMP_DEPT": "Manufacturing-Machin", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 79.44}, {"TNO": 40196, "ENAME": "TUSHAR LAXMANSINGH JAROLE", "EMP_DEPT": "Manufacturing-Machin", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 76.94}, {"TNO": 40192, "ENAME": "RAMESH RAGHUNATH ANAJI", "EMP_DEPT": "Manufacturing-Machin", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 76.17}, {"TNO": 40221, "ENAME": "SUNIL KUMAR MAURYA", "EMP_DEPT": "Manufacturing-Assemb", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 75.12}, {"TNO": 93260, "ENAME": "SWAPNIL EKNATH RAUT", "EMP_DEPT": "Manufacturing-Machin", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 72.15}, {"TNO": 40247, "ENAME": "PRADIP PANDURANG KALEKAR", "EMP_DEPT": "Manufacturing-Machin", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 70.93}, {"TNO": 40306, "ENAME": "DONDAPPA BASAVARAJ UDDANSHETTI", "EMP_DEPT": "Manufacturing-Assemb", "EMP_ORG_NAME": "ACD - PRODUCTS", "PERIOD_NAME": "APR-24", "PERFORMANCE_INDEX": 63.49}]</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>The top 10 employees with the highest performance index in April 2024 are:
+1. Sanket X Bhoite – 108.09
+2. Rajesh Vitthal Kute – 103.18
+3. Danish Dastagir Kazi – 100.88
+4. Nagesh Jagannath Boramani – 100.28
+5. Avdhut Maruti Desai – 100.00
+6. Akshay Rohidas Ladkat – 99.40
+7. Atif Aslam Maner – 97.63
+8. Nikhil Uttam Kambale – 96.87
+9. Akash Kashinath Nilaji – 96.71
+10. Shubham Chagan Khot – 96.27
+All these employees belong to the ACD - PRODUCTS organization, mainly within the Manufacturing-Machining and Manufacturing-Assembly departments.</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>normal_message</t>
+        </is>
+      </c>
+      <c r="AF6" t="inlineStr">
+        <is>
+          <t>fe179da0-aa84-44c2-b7c0-59a64177e903</t>
+        </is>
+      </c>
+      <c r="AG6" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update code with latest changes
</commit_message>
<xml_diff>
--- a/backend/data/New Flagged FAQ.xlsx
+++ b/backend/data/New Flagged FAQ.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG6"/>
+  <dimension ref="A1:AG8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1023,9 +1023,6 @@
           <t>Docket Employee Report</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>performance index more</t>
@@ -1079,8 +1076,6 @@
           <t>pending</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
           <t>thumbs_up</t>
@@ -1157,6 +1152,245 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>77cf0bb8b9e3b3985cb9c406eb87d670d84b32e715042b0fdb29df3bbdf56be8</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-10-27T07:22:10.844181+00:00</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Buyerwise OA Trolley Report</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>trolley ready for balancing</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>not ready for balancing</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>not ready for balancing</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Is the trolley not ready for balancing?</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>no_variables</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>[{"name": "org_name", "value": "ACD - CENTRI", "source": "option"}]</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>SELECT TROLLEY_NO, ORG_NAME, OA_NUMBER, SBM_NUMBER, TROLLEY_BALANCING_STATUS FROM KPCL_REPORTING.BUYERWISE_OA_TROLLEY_STATUS WHERE TROLLEY_BALANCING_STATUS LIKE 'Trolley not available to balance' AND BUYERWISE_OA_TROLLEY_STATUS.ORG_NAME LIKE '%{org_name}%';</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>SELECT TROLLEY_NO, ORG_NAME, OA_NUMBER, SBM_NUMBER, TROLLEY_BALANCING_STATUS FROM KPCL_REPORTING.BUYERWISE_OA_TROLLEY_STATUS WHERE TROLLEY_BALANCING_STATUS LIKE 'Trolley not available to balance' AND BUYERWISE_OA_TROLLEY_STATUS.ORG_NAME LIKE '%ACD - CENTRI%';</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
+        <v>50</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>ae812b85-23b3-46fa-8556-7d467aab4f58</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>14cbc80a-9599-4ed7-8da7-81c8cc3d4cc4</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>460ac0b9-7eab-4319-9903-0f9fa2ceadcc</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>modify</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>trolley ready for balancing</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>Is the trolley not ready for balancing?</t>
+        </is>
+      </c>
+      <c r="AB7" t="b">
+        <v>1</v>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>feedback</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>cc265b4d2ae93153387d274c9b4da0c0f87002c3e0ab9bc22dcbd986bcf5dbfb</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-10-27T09:45:44.214958+00:00</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Inventory Report</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>give me list of items safety stock whose consumption is not available from 3 years</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>SELECT ORG_NAME, CHILD_ITEM, CHILD_DESCRIPTION, SAFETY_STOCK FROM KPCL_REPORTING.FULLKIT_ITEMWISE_INV WHERE REQ_QTY_MONTH &lt; UPPER(TO_CHAR(SYSDATE, 'MON-YYYY')) AND NOT CHILD_ITEM LIKE 'N%' GROUP BY ORG_NAME, CHILD_ITEM, CHILD_DESCRIPTION, SAFETY_STOCK;</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>SELECT ORG_NAME, CHILD_ITEM, CHILD_DESCRIPTION, SAFETY_STOCK FROM KPCL_REPORTING.FULLKIT_ITEMWISE_INV WHERE REQ_QTY_MONTH &lt; UPPER(TO_CHAR(SYSDATE, 'MON-YYYY')) AND NOT CHILD_ITEM LIKE 'N%' GROUP BY ORG_NAME, CHILD_ITEM, CHILD_DESCRIPTION, SAFETY_STOCK;</t>
+        </is>
+      </c>
+      <c r="M8" t="n">
+        <v>50</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>d890c8e5-fff7-4f15-8c6b-336b99005da7</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>24f7bdb9-224b-48a2-b108-b004f30fe015</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>43681183-f6b2-426b-a4ce-cd3038c0956e</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>thumbs_down</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>down</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>give me list of items safety stock whose consumption is not available from 3 years</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>give me list of items safety stock whose consumption is not available from 3 years</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>adapt</t>
+        </is>
+      </c>
+      <c r="Z8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB8" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>[{"ORG_NAME": "PED - DEFENCE", "CHILD_ITEM": "999.02.878.50.", "CHILD_DESCRIPTION": "SCREW GRUB M8X1.25X12L", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - GEAR BOX", "CHILD_ITEM": "999.02.880.50.", "CHILD_DESCRIPTION": "SCREW GRUB M8X1.25X20L", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - DEFENCE", "CHILD_ITEM": "999.02.881.50.", "CHILD_DESCRIPTION": "SCREW GRUB M8X1.25X35L", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - DEFENCE", "CHILD_ITEM": "999.06.632.50.", "CHILD_DESCRIPTION": "NUT HEX M10X1.5P", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - DEFENCE", "CHILD_ITEM": "999.06.669.50.", "CHILD_DESCRIPTION": "NUT HEX M14X2", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "ACD - SPARES", "CHILD_ITEM": "999.06.687.50.", "CHILD_DESCRIPTION": "NUT HEX, M16 X 2P", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - GEAR BOX", "CHILD_ITEM": "999.06.742.50.", "CHILD_DESCRIPTION": "NUT HEX M20X2.5", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - GEAR BOX", "CHILD_ITEM": "999.11.262.50.", "CHILD_DESCRIPTION": "WASHER, SPRING, ID 8.2 X THK 2.0", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - GEAR BOX", "CHILD_ITEM": "999.11.274.50.", "CHILD_DESCRIPTION": "WASHER SPRING ID12.2X2.5 mm", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - GEAR BOX", "CHILD_ITEM": "649.07.604.50.", "CHILD_DESCRIPTION": "KEY PARALLEL ROUND END 28X16X130 CH", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - GEAR BOX", "CHILD_ITEM": "650.14.003.50.", "CHILD_DESCRIPTION": "RING", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - DEFENCE", "CHILD_ITEM": "999.01.702.50.", "CHILD_DESCRIPTION": "BOLT HEX STD M16X2X100L E", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - DEFENCE", "CHILD_ITEM": "999.01.715.50.", "CHILD_DESCRIPTION": "SCREW HEX STD M16X2X55L", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - DEFENCE", "CHILD_ITEM": "999.01.752.50.", "CHILD_DESCRIPTION": "BOLT HEX STD M20X2.5X65L E", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - DEFENCE", "CHILD_ITEM": "999.02.372.00.", "CHILD_DESCRIPTION": "SCREW SOCK STD 5/16XUNCX1L", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - DEFENCE", "CHILD_ITEM": "999.02.701.50.", "CHILD_DESCRIPTION": "SCREW SOCKET STD, M16 X 2 X 45L", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - DEFENCE", "CHILD_ITEM": "999.02.788.50.", "CHILD_DESCRIPTION": "SCREW SOCK STD M5X0.8X16L", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "ACD - SPARES", "CHILD_ITEM": "35.256.310.00.", "CHILD_DESCRIPTION": "GLASS SIGHT (TOUGHENED GLASS) FOR 2 \"BSP WATER FLOW INDICATOR / /", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "ACD - SPARES", "CHILD_ITEM": "35.262.240.00.", "CHILD_DESCRIPTION": "GUIDE FOR REGULATING TABLE OF 70CR51 SUCTION VALVE, EN-56", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - GEAR BOX", "CHILD_ITEM": "500.14.432.50.", "CHILD_DESCRIPTION": "SET OF HEIGHT BLOCK FOR BHEL STAND-300X250X18.6THK", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - GEAR BOX", "CHILD_ITEM": "999.11.523.50.", "CHILD_DESCRIPTION": "WASHER SPRING STEEL PLATING ID12.2X 2.5TH", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - GEAR BOX", "CHILD_ITEM": "999.12.515.00.", "CHILD_DESCRIPTION": "O RING CORD DIA 5.00 NEO PRENE", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - GEAR BOX", "CHILD_ITEM": "999.12.693.50.", "CHILD_DESCRIPTION": "O RING VITO - X36.500X3.000 0XC", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - GEAR BOX", "CHILD_ITEM": "999.16.009.50.", "CHILD_DESCRIPTION": "FERRULE ID10 STEEL", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - GEAR BOX", "CHILD_ITEM": "650.17.205.50.", "CHILD_DESCRIPTION": "SPACER", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - GEAR BOX", "CHILD_ITEM": "650.17.212.50.", "CHILD_DESCRIPTION": "KEY PARALLEL SQ.END 50x28x170", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - GEAR BOX", "CHILD_ITEM": "650.17.214.50.", "CHILD_DESCRIPTION": "SPACER", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - GEAR BOX", "CHILD_ITEM": "650.17.216.50.", "CHILD_DESCRIPTION": "SEAL FACE V", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - GEAR BOX", "CHILD_ITEM": "650.17.619.50.", "CHILD_DESCRIPTION": "OIL CATCHER", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - DEFENCE", "CHILD_ITEM": "999.09.758.50.", "CHILD_DESCRIPTION": "DOWEL PIN, DIA 12 X 40L, 141 CITY", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - DEFENCE", "CHILD_ITEM": "999.09.782.50.", "CHILD_DESCRIPTION": "CYLINDRICAL PIN DIA16.00X40L E", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "ACD - SCREW", "CHILD_ITEM": "999.11.274.50.", "CHILD_DESCRIPTION": "WASHER SPRING ID12.2X2.5 mm", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - DEFENCE", "CHILD_ITEM": "999.11.280.50.", "CHILD_DESCRIPTION": "WASHER, SPRING, ID 14.2 X THK 3.0", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - GEAR BOX", "CHILD_ITEM": "503.00.130.00.", "CHILD_DESCRIPTION": "ASSLY FILTER ELEMENT (CH)", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - GEAR BOX", "CHILD_ITEM": "503.00.205.00.", "CHILD_DESCRIPTION": "RING PISTON 3\" DIA CLUTCH", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - DEFENCE", "CHILD_ITEM": "503.01.809.00.", "CHILD_DESCRIPTION": "PLUG 1-11 1/2NPTF (CH)", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - DEFENCE", "CHILD_ITEM": "516.00.605.00.", "CHILD_DESCRIPTION": "CONNECTOR (1/2\"NPTF X 1/2\"BSP)", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "ACD - CENTRI", "CHILD_ITEM": "61.800.084.00.", "CHILD_DESCRIPTION": "CABLE TRAY, GI PERFORATED, 150 x 50 WITH COVER (SPEC. NO.- SP-EL-659).", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - DEFENCE", "CHILD_ITEM": "999.18.422.50.", "CHILD_DESCRIPTION": "WASHER PLAIN COPPER 26.3X2", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - DEFENCE", "CHILD_ITEM": "999.21.109.50.", "CHILD_DESCRIPTION": "NUT LOCK M140X2 SKF KM28", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - GEAR BOX", "CHILD_ITEM": "650.18.810.66.", "CHILD_DESCRIPTION": "Parallel Pin ISO 8735 - 16x60-B - St", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - GEAR BOX", "CHILD_ITEM": "650.19.170.02.", "CHILD_DESCRIPTION": "PLATE NAME BLANK", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - GEAR BOX", "CHILD_ITEM": "650.21.529.50.", "CHILD_DESCRIPTION": "SCREW HEX HD M24X3X110", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - GEAR BOX", "CHILD_ITEM": "650.88.730.03.", "CHILD_DESCRIPTION": "KEY PARALLEL 25X14X110L CH", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - GEAR BOX", "CHILD_ITEM": "653.11.920.04.", "CHILD_DESCRIPTION": "PLATE OIL SEAL RETAINER", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - GEAR BOX", "CHILD_ITEM": "653.15.810.34.", "CHILD_DESCRIPTION": "AIR VENT 1/4\"", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - GEAR BOX", "CHILD_ITEM": "653.18.950.04.", "CHILD_DESCRIPTION": "KEY PARALLEL SQ END (14X9X25)", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - GEAR BOX", "CHILD_ITEM": "653.21.550.06.", "CHILD_DESCRIPTION": "PLATE RETAINER M.S.", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - DEFENCE", "CHILD_ITEM": "999.11.298.50.", "CHILD_DESCRIPTION": "WASHER SPRING ID20.2X4 mm", "SAFETY_STOCK": 0.0}, {"ORG_NAME": "PED - DEFENCE", "CHILD_ITEM": "999.13.679.50.", "CHILD_DESCRIPTION": "CIRCLIP EXTERNAL TYPE A 190X4.000TH K", "SAFETY_STOCK": 0.0}]</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>There are 50 items listed with safety stock values, all showing zero safety stock. These items have no recorded consumption for the past 3 years. You can review the full list of these items and their descriptions in the table.</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>normal_message</t>
+        </is>
+      </c>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>aff8181f-8d9f-44a8-8f9c-8cf59e91b2d9</t>
+        </is>
+      </c>
+      <c r="AG8" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>